<commit_message>
Updated code and output Jul 30
</commit_message>
<xml_diff>
--- a/output_python/02_make_meta2.ipynb/metadata_count_purity.xlsx
+++ b/output_python/02_make_meta2.ipynb/metadata_count_purity.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R50"/>
+  <dimension ref="A1:R51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2804,42 +2804,30 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>TWJF-10146-MO011-9999_TEST</t>
+          <t>TWJF-5120-15</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Metastatic TNBC</t>
+          <t>Pancreas</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>CTEP</t>
+          <t>Leidos/NCI</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>BARD1,BRCA2,RB1,TP53</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/CTEP/analysis/TWJF-10146-MO011-0029/itb-review-files/10146-0029.Annotated.Neoantigen_Candidates.Revd.tsv</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/CTEP/analysis/TWJF-10146-MO011-0029/gcp_immuno/final_results/pVACseq/mhc_i/TWJF-10146-0029-0029_Tumor_Lysate.all_epitopes.tsv</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/CTEP/analysis/TWJF-10146-MO011-0029/gcp_immuno/final_results/pVACseq/mhc_ii/TWJF-10146-0029-0029_Tumor_Lysate.all_epitopes.aggregated.tsv</t>
-        </is>
-      </c>
+          <t>TP53,ACVR1B,ACVR2A,AKT2,APC,ATRX,BRAF,BRCA2,DAXX,ELF3,EP300,FAT1,FAT4,GNAS,HIF1A,KRAS,MAP2K4,MEN1,PREX2,RNF43,SMAD4,SND1,STK11</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
-          <t>A duplicate of TWJF-10146-MO011-0029, but changed the ID name for testing purpose</t>
+          <t>screen fail</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2849,44 +2837,22 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K33" t="n">
-        <v>62</v>
-      </c>
-      <c r="L33" t="n">
-        <v>6</v>
-      </c>
-      <c r="M33" t="n">
-        <v>12</v>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>chr1-114677966-114677967-G-T</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>AMPD1</t>
-        </is>
-      </c>
-      <c r="P33" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R33" t="n">
-        <v>0.9399999999999999</v>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>TWJF-5120-15</t>
+          <t>TWJF-5120-16</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2904,14 +2870,24 @@
           <t>TP53,ACVR1B,ACVR2A,AKT2,APC,ATRX,BRAF,BRCA2,DAXX,ELF3,EP300,FAT1,FAT4,GNAS,HIF1A,KRAS,MAP2K4,MEN1,PREX2,RNF43,SMAD4,SND1,STK11</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>screen fail</t>
-        </is>
-      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analysis/TWJF-5120-16/itb-review-files/5120-16.Annotated.Neoantigen_Candidates.tsv</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analy
+sis/TWJF-5120-16/gcp_immuno/final_results/pVACseq/mhc_i/5120_16_Tumor_FF.all_epitopes.tsv</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analy
+sis/TWJF-5120-16/gcp_immuno/final_results/pVACseq/mhc_ii/5120_16_Tumor_FF.all_epitopes.aggregated.tsv</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
           <t>No</t>
@@ -2919,22 +2895,44 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K34" t="n">
+        <v>32</v>
+      </c>
+      <c r="L34" t="n">
+        <v>8</v>
+      </c>
+      <c r="M34" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>chr12-25245349-25245350-C-T</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>KRAS</t>
+        </is>
+      </c>
+      <c r="P34" t="n">
+        <v>0.147</v>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="R34" t="n">
+        <v>0.294</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>TWJF-5120-16</t>
+          <t>TWJF-5120-19</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2954,103 +2952,103 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analysis/TWJF-5120-16/itb-review-files/5120-16.Annotated.Neoantigen_Candidates.tsv</t>
+          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analysis/TWJF-5120-19/itb-review-files/5120-19.Annotated.Neoantigen_Candidates.tsv</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
-        <is>
-          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analy
-sis/TWJF-5120-16/gcp_immuno/final_results/pVACseq/mhc_i/5120_16_Tumor_FF.all_epitopes.tsv</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analy
-sis/TWJF-5120-16/gcp_immuno/final_results/pVACseq/mhc_ii/5120_16_Tumor_FF.all_epitopes.aggregated.tsv</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K35" t="n">
-        <v>32</v>
-      </c>
-      <c r="L35" t="n">
-        <v>8</v>
-      </c>
-      <c r="M35" t="n">
-        <v>0</v>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>chr12-25245349-25245350-C-T</t>
-        </is>
-      </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>KRAS</t>
-        </is>
-      </c>
-      <c r="P35" t="n">
-        <v>0.147</v>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="R35" t="n">
-        <v>0.294</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>TWJF-5120-19</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Pancreas</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Leidos/NCI</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>TP53,ACVR1B,ACVR2A,AKT2,APC,ATRX,BRAF,BRCA2,DAXX,ELF3,EP300,FAT1,FAT4,GNAS,HIF1A,KRAS,MAP2K4,MEN1,PREX2,RNF43,SMAD4,SND1,STK11</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analysis/TWJF-5120-19/itb-review-files/5120-19.Annotated.Neoantigen_Candidates.tsv</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
         <is>
           <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pa
 ncreas_leidos/analysis/TWJF-5120-19/gcp_immuno/final_results_v3_relaxed_var_filters/pVACseq/mhc_i/5120_1
 9_Tumor_FF.all_epitopes.tsv</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pa
 ncreas_leidos/analysis/TWJF-5120-19/gcp_immuno/final_results_v3_relaxed_var_filters/pVACseq/mhc_ii/5120_
 19_Tumor_FF.all_epitopes.aggregated.tsv</t>
         </is>
       </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K35" t="n">
+        <v>30</v>
+      </c>
+      <c r="L35" t="n">
+        <v>5</v>
+      </c>
+      <c r="M35" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>chr17-7675087-7675088-C-T</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>TP53</t>
+        </is>
+      </c>
+      <c r="P35" t="n">
+        <v>0.07099999999999999</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="R35" t="n">
+        <v>0.142</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>TWJF-5120-17</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Pancreas</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Leidos/NCI</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>TP53,ACVR1B,ACVR2A,AKT2,APC,ATRX,BRAF,BRCA2,DAXX,ELF3,EP300,FAT1,FAT4,GNAS,HIF1A,KRAS,MAP2K4,MEN1,PREX2,RNF43,SMAD4,SND1,STK12</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analysis/TWJF-5120-17/itb-review-files/5120-17.Annotated.Neoantigen_Candidates.tsv</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos
+/analysis/TWJF-5120-17/gcp_immuno/final_results/pVACseq/mhc_i/5120-17-Tumor-FF.all_epitopes.tsv</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos
+/analysis/TWJF-5120-17/gcp_immuno/final_results/pVACseq/mhc_ii/5120-17-Tumor-FF.all_epitopes.aggregated.tsv</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
@@ -3063,26 +3061,26 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>30</v>
+        <v>85</v>
       </c>
       <c r="L36" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M36" t="n">
         <v>0</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>chr17-7675087-7675088-C-T</t>
+          <t>chr12-25245349-25245350-C-T</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>TP53</t>
+          <t>KRAS</t>
         </is>
       </c>
       <c r="P36" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.405</v>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
@@ -3090,13 +3088,13 @@
         </is>
       </c>
       <c r="R36" t="n">
-        <v>0.142</v>
+        <v>0.8100000000000001</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TWJF-5120-17</t>
+          <t>TWJF-5120-18</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3111,109 +3109,111 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>TP53,ACVR1B,ACVR2A,AKT2,APC,ATRX,BRAF,BRCA2,DAXX,ELF3,EP300,FAT1,FAT4,GNAS,HIF1A,KRAS,MAP2K4,MEN1,PREX2,RNF43,SMAD4,SND1,STK12</t>
+          <t>TP53,ACVR1B,ACVR2A,AKT2,APC,ATRX,BRAF,BRCA2,DAXX,ELF3,EP300,FAT1,FAT4,GNAS,HIF1A,KRAS,MAP2K4,MEN1,PREX2,RNF43,SMAD4,SND1,STK13</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analysis/TWJF-5120-17/itb-review-files/5120-17.Annotated.Neoantigen_Candidates.tsv</t>
+          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analysis/TWJF-5120-18/itb-review-files/5120-18.Annotated.Neoantigen_Candidates.tsv</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
-        <is>
-          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos
-/analysis/TWJF-5120-17/gcp_immuno/final_results/pVACseq/mhc_i/5120-17-Tumor-FF.all_epitopes.tsv</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos
-/analysis/TWJF-5120-17/gcp_immuno/final_results/pVACseq/mhc_ii/5120-17-Tumor-FF.all_epitopes.aggregated.tsv</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K37" t="n">
-        <v>85</v>
-      </c>
-      <c r="L37" t="n">
-        <v>1</v>
-      </c>
-      <c r="M37" t="n">
-        <v>0</v>
-      </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>chr12-25245349-25245350-C-T</t>
-        </is>
-      </c>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t>KRAS</t>
-        </is>
-      </c>
-      <c r="P37" t="n">
-        <v>0.405</v>
-      </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="R37" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>TWJF-5120-18</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Pancreas</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Leidos/NCI</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>TP53,ACVR1B,ACVR2A,AKT2,APC,ATRX,BRAF,BRCA2,DAXX,ELF3,EP300,FAT1,FAT4,GNAS,HIF1A,KRAS,MAP2K4,MEN1,PREX2,RNF43,SMAD4,SND1,STK13</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analysis/TWJF-5120-18/itb-review-files/5120-18.Annotated.Neoantigen_Candidates.tsv</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
         <is>
           <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pa
 ncreas_leidos/analysis/TWJF-5120-18/gcp_immuno/final_results/pVACseq/mhc_i/5120_18_Tumor_FF.all_epitopes
 .tsv</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pa
 ncreas_leidos/analysis/TWJF-5120-18/gcp_immuno/final_results/pVACseq/mhc_ii/5120_18_Tumor_FF.all_epitope
 s.aggregated.tsv</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K37" t="n">
+        <v>23</v>
+      </c>
+      <c r="L37" t="n">
+        <v>3</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>chr12-25245349-25245350-C-T</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>KRAS</t>
+        </is>
+      </c>
+      <c r="P37" t="n">
+        <v>0.113</v>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="R37" t="n">
+        <v>0.226</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>5120-39</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Pancreas</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Leidos/NCI</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>TP53,ACVR1B,ACVR2A,AKT2,APC,ATRX,BRAF,BRCA2,DAXX,ELF3,EP300,FAT1,FAT4,GNAS,HIF1A,KRAS,MAP2K4,MEN1,PREX2,RNF43,SMAD4,SND1,STK14</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analysis/TWJF-5120-39/itb-review-files/Leidos-39.Annotated.Neoantigen_Candidates.tsv</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analysis/TWJF-5120-39/gcp_immuno/final_results/pVACseq/mhc_i/5120-39-TumorDNA.all_epitopes.tsv</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analysis/TWJF-5120-39/gcp_immuno/final_results/pVACseq/mhc_ii/5120-39-TumorDNA.all_epitopes.aggregated.tsv</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Video analysis: before prediction</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr">
         <is>
           <t>No</t>
@@ -3225,17 +3225,17 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="L38" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M38" t="n">
         <v>0</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>chr12-25245349-25245350-C-T</t>
+          <t>chr12-25227341-25227342-T-C</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
@@ -3244,7 +3244,7 @@
         </is>
       </c>
       <c r="P38" t="n">
-        <v>0.113</v>
+        <v>0.414</v>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
@@ -3252,46 +3252,50 @@
         </is>
       </c>
       <c r="R38" t="n">
-        <v>0.226</v>
+        <v>0.828</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>5120-39</t>
+          <t>CTEP-10146-MD017-0052</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Pancreas</t>
+          <t>Metastatic TNBC</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Leidos/NCI</t>
+          <t>CTEP</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>TP53,ACVR1B,ACVR2A,AKT2,APC,ATRX,BRAF,BRCA2,DAXX,ELF3,EP300,FAT1,FAT4,GNAS,HIF1A,KRAS,MAP2K4,MEN1,PREX2,RNF43,SMAD4,SND1,STK14</t>
+          <t>BARD1,BRCA2,RB1,TP53</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analysis/TWJF-5120-39/itb-review-files/Leidos-39.Annotated.Neoantigen_Candidates.tsv</t>
+          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/CTEP/analysis/10146-0052/itb-review-files/CTEP-52.Annotated.Neoantigen_Candidates.tsv</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analysis/TWJF-5120-39/gcp_immuno/final_results/pVACseq/mhc_i/5120-39-TumorDNA.all_epitopes.tsv</t>
+          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/CTEP/analysis/10146-0052/gcp_immuno/final_results/pVACseq/mhc_i/10146_0052_Tumor_Lysate.all_epitopes.tsv</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analysis/TWJF-5120-39/gcp_immuno/final_results/pVACseq/mhc_ii/5120-39-TumorDNA.all_epitopes.aggregated.tsv</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr"/>
+          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/CTEP/analysis/10146-0052/gcp_immuno/final_results/pVACseq/mhc_ii/10146_0052_Tumor_Lysate.all_epitopes.aggregated.tsv</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Video analysis: before prediction</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
           <t>No</t>
@@ -3303,26 +3307,26 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>35</v>
+        <v>72</v>
       </c>
       <c r="L39" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M39" t="n">
         <v>0</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>chr12-25227341-25227342-T-C</t>
+          <t>chr17-7674887-7674888-T-C</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>KRAS</t>
+          <t>TP53</t>
         </is>
       </c>
       <c r="P39" t="n">
-        <v>0.414</v>
+        <v>0.419</v>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
@@ -3330,46 +3334,46 @@
         </is>
       </c>
       <c r="R39" t="n">
-        <v>0.828</v>
+        <v>0.838</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CTEP-10146-MD017-0052</t>
+          <t>G110_Region1</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Metastatic TNBC</t>
+          <t>Glioblastoma</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>CTEP</t>
+          <t>Johanns</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>BARD1,BRCA2,RB1,TP53</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/CTEP/analysis/10146-0052/itb-review-files/CTEP-52.Annotated.Neoantigen_Candidates.tsv</t>
-        </is>
-      </c>
+          <t>TP53,DAXX,GOPC,HIF1A,IDH1,IDH2,LZTR1,MDM4,PDGFRA,PIK3CA,PIK3R1,PTPRD,ROS1,SALL4,STAG2,TERT</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
-          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/CTEP/analysis/10146-0052/gcp_immuno/final_results/pVACseq/mhc_i/10146_0052_Tumor_Lysate.all_epitopes.tsv</t>
+          <t>/storage1/fs1/gpdunn/Active/Project_0001_Clinical/gc2609/gbm_antigen_dunn/vaccine_G110/gcp_immuno_region1/final_results/pVACseq/mhc_i/TumorDNA-G110_Region1.all_epitopes.aggregated.tsv</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>/storage1/fs1/gillandersw/Active/Project_0001_Clinical_Trials/CTEP/analysis/10146-0052/gcp_immuno/final_results/pVACseq/mhc_ii/10146_0052_Tumor_Lysate.all_epitopes.aggregated.tsv</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr"/>
+          <t>/storage1/fs1/gpdunn/Active/Project_0001_Clinical/gc2609/gbm_antigen_dunn/vaccine_G110/gcp_immuno_region1/final_results/pVACseq/mhc_ii/TumorDNA-G110_Region1.all_epitopes.aggregated.tsv</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>This case involved sequencing of 2 regions of a brain tumor.</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
           <t>No</t>
@@ -3377,44 +3381,38 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K40" t="n">
-        <v>72</v>
-      </c>
-      <c r="L40" t="n">
-        <v>1</v>
-      </c>
-      <c r="M40" t="n">
-        <v>0</v>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr">
         <is>
-          <t>chr17-7674887-7674888-T-C</t>
+          <t>chr10-87894102-87894103-T-C</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>TP53</t>
+          <t>PTEN</t>
         </is>
       </c>
       <c r="P40" t="n">
-        <v>0.419</v>
+        <v>0.41</v>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="R40" t="n">
-        <v>0.838</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>G110_Region1</t>
+          <t>G110_Region2</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3435,19 +3433,15 @@
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
-          <t>/storage1/fs1/gpdunn/Active/Project_0001_Clinical/gc2609/gbm_antigen_dunn/vaccine_G110/gcp_immuno_region1/final_results/pVACseq/mhc_i/TumorDNA-G110_Region1.all_epitopes.aggregated.tsv</t>
+          <t>/storage1/fs1/gpdunn/Active/Project_0001_Clinical/gc2609/gbm_antigen_dunn/vaccine_G110/gcp_immuno_region2/final_results/pVACseq/mhc_i/TumorDNA-G110_Region2.all_epitopes.aggregated.tsv</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>/storage1/fs1/gpdunn/Active/Project_0001_Clinical/gc2609/gbm_antigen_dunn/vaccine_G110/gcp_immuno_region1/final_results/pVACseq/mhc_ii/TumorDNA-G110_Region1.all_epitopes.aggregated.tsv</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>This case involved sequencing of 2 regions of a brain tumor.</t>
-        </is>
-      </c>
+          <t>/storage1/fs1/gpdunn/Active/Project_0001_Clinical/gc2609/gbm_antigen_dunn/vaccine_G110/gcp_immuno_region2/final_results/pVACseq/mhc_ii/TumorDNA-G110_Region2.all_epitopes.aggregated.tsv</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
           <t>No</t>
@@ -3455,18 +3449,12 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K41" t="n">
-        <v>58</v>
-      </c>
-      <c r="L41" t="n">
-        <v>4</v>
-      </c>
-      <c r="M41" t="n">
-        <v>0</v>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr">
         <is>
           <t>chr10-87894102-87894103-T-C</t>
@@ -3478,7 +3466,7 @@
         </is>
       </c>
       <c r="P41" t="n">
-        <v>0.41</v>
+        <v>0.35</v>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
@@ -3486,13 +3474,13 @@
         </is>
       </c>
       <c r="R41" t="n">
-        <v>0.82</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>G110_Region2</t>
+          <t>G113_Region1</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3513,12 +3501,12 @@
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
-          <t>/storage1/fs1/gpdunn/Active/Project_0001_Clinical/gc2609/gbm_antigen_dunn/vaccine_G110/gcp_immuno_region2/final_results/pVACseq/mhc_i/TumorDNA-G110_Region2.all_epitopes.aggregated.tsv</t>
+          <t>/storage1/fs1/gpdunn/Active/Project_0001_Clinical/gc2609/gbm_antigen_dunn/vaccine_G113/gcp_immuno_region1/final_results/pVACseq/mhc_i/TumorDNA-G113_Region1.all_epitopes.aggregated.tsv</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>/storage1/fs1/gpdunn/Active/Project_0001_Clinical/gc2609/gbm_antigen_dunn/vaccine_G110/gcp_immuno_region2/final_results/pVACseq/mhc_ii/TumorDNA-G110_Region2.all_epitopes.aggregated.tsv</t>
+          <t>/storage1/fs1/gpdunn/Active/Project_0001_Clinical/gc2609/gbm_antigen_dunn/vaccine_G113/gcp_immuno_region1/final_results/pVACseq/mhc_ii/TumorDNA-G113_Region1.all_epitopes.aggregated.tsv</t>
         </is>
       </c>
       <c r="H42" t="inlineStr"/>
@@ -3529,30 +3517,24 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K42" t="n">
-        <v>48</v>
-      </c>
-      <c r="L42" t="n">
-        <v>3</v>
-      </c>
-      <c r="M42" t="n">
-        <v>0</v>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr">
         <is>
-          <t>chr10-87894102-87894103-T-C</t>
+          <t>chr11-123939725-123939726-T-C</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>OR4D5</t>
         </is>
       </c>
       <c r="P42" t="n">
-        <v>0.35</v>
+        <v>0.497</v>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
@@ -3560,13 +3542,13 @@
         </is>
       </c>
       <c r="R42" t="n">
-        <v>0.7</v>
+        <v>0.994</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>G113_Region1</t>
+          <t>G113_Region2</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3587,15 +3569,19 @@
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
-          <t>/storage1/fs1/gpdunn/Active/Project_0001_Clinical/gc2609/gbm_antigen_dunn/vaccine_G113/gcp_immuno_region1/final_results/pVACseq/mhc_i/TumorDNA-G113_Region1.all_epitopes.aggregated.tsv</t>
+          <t>/storage1/fs1/gpdunn/Active/Project_0001_Clinical/gc2609/gbm_antigen_dunn/vaccine_G113/gcp_immuno_region2/final_results/pVACseq/mhc_i/TumorDNA-G113_Region2.all_epitopes.aggregated.tsv</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>/storage1/fs1/gpdunn/Active/Project_0001_Clinical/gc2609/gbm_antigen_dunn/vaccine_G113/gcp_immuno_region1/final_results/pVACseq/mhc_ii/TumorDNA-G113_Region1.all_epitopes.aggregated.tsv</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr"/>
+          <t>/storage1/fs1/gpdunn/Active/Project_0001_Clinical/gc2609/gbm_antigen_dunn/vaccine_G113/gcp_immuno_region2/final_results/pVACseq/mhc_ii/TumorDNA-G113_Region2.all_epitopes.aggregated.tsv</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Seems to have too many marked with "Pending" after ITB review, excluded</t>
+        </is>
+      </c>
       <c r="I43" t="inlineStr">
         <is>
           <t>No</t>
@@ -3603,30 +3589,24 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K43" t="n">
-        <v>33</v>
-      </c>
-      <c r="L43" t="n">
-        <v>5</v>
-      </c>
-      <c r="M43" t="n">
-        <v>0</v>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr">
         <is>
-          <t>chr11-123939725-123939726-T-C</t>
+          <t>chr16-31297551-31297552-C-T</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>OR4D5</t>
+          <t>ITGAM</t>
         </is>
       </c>
       <c r="P43" t="n">
-        <v>0.497</v>
+        <v>0.486</v>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
@@ -3634,44 +3614,44 @@
         </is>
       </c>
       <c r="R43" t="n">
-        <v>0.994</v>
+        <v>0.972</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>G113_Region2</t>
+          <t>TWJF-5120-41</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Glioblastoma</t>
+          <t>Pancreas</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Johanns</t>
+          <t>Leidos/NCI</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>TP53,DAXX,GOPC,HIF1A,IDH1,IDH2,LZTR1,MDM4,PDGFRA,PIK3CA,PIK3R1,PTPRD,ROS1,SALL4,STAG2,TERT</t>
+          <t>TP53,ACVR1B,ACVR2A,AKT2,APC,ATRX,BRAF,BRCA2,DAXX,ELF3,EP300,FAT1,FAT4,GNAS,HIF1A,KRAS,MAP2K4,MEN1,PREX2,RNF43,SMAD4,SND1,STK11</t>
         </is>
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
-          <t>/storage1/fs1/gpdunn/Active/Project_0001_Clinical/gc2609/gbm_antigen_dunn/vaccine_G113/gcp_immuno_region2/final_results/pVACseq/mhc_i/TumorDNA-G113_Region2.all_epitopes.aggregated.tsv</t>
+          <t>/Volumes/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analysis/TWJF-5120-41/gcp_immuno/final_results/pVACseq/mhc_i/5120-41-TumorDNA.all_epitopes.tsv</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>/storage1/fs1/gpdunn/Active/Project_0001_Clinical/gc2609/gbm_antigen_dunn/vaccine_G113/gcp_immuno_region2/final_results/pVACseq/mhc_ii/TumorDNA-G113_Region2.all_epitopes.aggregated.tsv</t>
+          <t>/Volumes/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analysis/TWJF-5120-41/gcp_immuno/final_results/pVACseq/mhc_ii/5120-41-TumorDNA.all_epitopes.aggregated.tsv</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Seems to have too many marked with "Pending" after ITB review, excluded</t>
+          <t>Video analysis: before prediction</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3681,38 +3661,44 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K44" t="n">
+        <v>48</v>
+      </c>
+      <c r="L44" t="n">
+        <v>0</v>
+      </c>
+      <c r="M44" t="n">
+        <v>0</v>
+      </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>chr16-31297551-31297552-C-T</t>
+          <t>chr17-7673775-7673776-G-A</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>ITGAM</t>
+          <t>TP53</t>
         </is>
       </c>
       <c r="P44" t="n">
-        <v>0.486</v>
+        <v>0.287</v>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="R44" t="n">
-        <v>0.972</v>
+        <v>0.574</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>TWJF-5120-41</t>
+          <t>TWJF-5120-42</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3733,15 +3719,19 @@
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
-          <t>/Volumes/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analysis/TWJF-5120-41/gcp_immuno/final_results/pVACseq/mhc_i/5120-41-TumorDNA.all_epitopes.tsv</t>
+          <t>/Volumes/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analysis/TWJF-5120-42/gcp_immuno/final_results/pVACseq/mhc_i/5120-42-TumorDNA.all_epitopes.tsv</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>/Volumes/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analysis/TWJF-5120-41/gcp_immuno/final_results/pVACseq/mhc_ii/5120-41-TumorDNA.all_epitopes.aggregated.tsv</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr"/>
+          <t>/Volumes/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analysis/TWJF-5120-42/gcp_immuno/final_results/pVACseq/mhc_ii/5120-42-TumorDNA.all_epitopes.aggregated.tsv</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Video analysis: before prediction</t>
+        </is>
+      </c>
       <c r="I45" t="inlineStr">
         <is>
           <t>No</t>
@@ -3753,17 +3743,17 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="L45" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="M45" t="n">
         <v>0</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>chr17-7673775-7673776-G-A</t>
+          <t>chr17-7673805-7673806-C-A</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
@@ -3772,7 +3762,7 @@
         </is>
       </c>
       <c r="P45" t="n">
-        <v>0.287</v>
+        <v>0.306</v>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
@@ -3780,42 +3770,46 @@
         </is>
       </c>
       <c r="R45" t="n">
-        <v>0.574</v>
+        <v>0.612</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>TWJF-5120-42</t>
+          <t>10146-0053</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Pancreas</t>
+          <t>Metastatic TNBC</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Leidos/NCI</t>
+          <t>CTEP</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>TP53,ACVR1B,ACVR2A,AKT2,APC,ATRX,BRAF,BRCA2,DAXX,ELF3,EP300,FAT1,FAT4,GNAS,HIF1A,KRAS,MAP2K4,MEN1,PREX2,RNF43,SMAD4,SND1,STK11</t>
+          <t>BARD1,BRCA2,RB1,TP53</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
-          <t>/Volumes/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analysis/TWJF-5120-42/gcp_immuno/final_results/pVACseq/mhc_i/5120-42-TumorDNA.all_epitopes.tsv</t>
+          <t>/Volumes/gillandersw/Active/Project_0001_Clinical_Trials/CTEP/analysis/10146-FL507-0053/gcp_immuno/final_results/pVACseq/mhc_i/10146-0053-TumorDNA.all_epitopes.tsv</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>/Volumes/gillandersw/Active/Project_0001_Clinical_Trials/pancreas_leidos/analysis/TWJF-5120-42/gcp_immuno/final_results/pVACseq/mhc_ii/5120-42-TumorDNA.all_epitopes.aggregated.tsv</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr"/>
+          <t>/Volumes/gillandersw/Active/Project_0001_Clinical_Trials/CTEP/analysis/10146-FL507-0053/gcp_immuno/final_results/pVACseq/mhc_ii/10146-0053-TumorDNA.all_epitopes.aggregated.tsv</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Video analysis: after prediction revealed</t>
+        </is>
+      </c>
       <c r="I46" t="inlineStr">
         <is>
           <t>No</t>
@@ -3827,40 +3821,40 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="L46" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="M46" t="n">
         <v>0</v>
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>chr17-7673805-7673806-C-A</t>
+          <t>chr6-44255310-44255311-G-C</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>TP53</t>
+          <t>SLC35B2</t>
         </is>
       </c>
       <c r="P46" t="n">
-        <v>0.306</v>
+        <v>0.472</v>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="R46" t="n">
-        <v>0.612</v>
+        <v>0.944</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>10146-0053</t>
+          <t>10146-0054</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3881,15 +3875,19 @@
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
-          <t>/Volumes/gillandersw/Active/Project_0001_Clinical_Trials/CTEP/analysis/10146-FL507-0053/gcp_immuno/final_results/pVACseq/mhc_i/10146-0053-TumorDNA.all_epitopes.tsv</t>
+          <t>/Volumes/gillandersw/Active/Project_0001_Clinical_Trials/CTEP/analysis/10146-CO070-0054/gcp_immuno/final_results/pVACseq/mhc_i/10146-0054-TumorDNA.all_epitopes.tsv</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>/Volumes/gillandersw/Active/Project_0001_Clinical_Trials/CTEP/analysis/10146-FL507-0053/gcp_immuno/final_results/pVACseq/mhc_ii/10146-0053-TumorDNA.all_epitopes.aggregated.tsv</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr"/>
+          <t>/Volumes/gillandersw/Active/Project_0001_Clinical_Trials/CTEP/analysis/10146-CO070-0054/gcp_immuno/final_results/pVACseq/mhc_ii/10146-0054-TumorDNA.all_epitopes.aggregated.tsv</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Video analysis: after prediction revealed</t>
+        </is>
+      </c>
       <c r="I47" t="inlineStr">
         <is>
           <t>No</t>
@@ -3901,26 +3899,26 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L47" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="M47" t="n">
         <v>0</v>
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>chr6-44255310-44255311-G-C</t>
+          <t>chr20-64105860-64105861-C-T</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>SLC35B2</t>
+          <t>NPBWR2</t>
         </is>
       </c>
       <c r="P47" t="n">
-        <v>0.472</v>
+        <v>0.482</v>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
@@ -3928,42 +3926,38 @@
         </is>
       </c>
       <c r="R47" t="n">
-        <v>0.944</v>
+        <v>0.964</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>10146-0054</t>
+          <t>04143-004</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Metastatic TNBC</t>
+          <t>SCLC</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>CTEP</t>
+          <t>Ward</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>BARD1,BRCA2,RB1,TP53</t>
+          <t>FAM135B,RB1,TP53</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>/Volumes/gillandersw/Active/Project_0001_Clinical_Trials/CTEP/analysis/10146-CO070-0054/gcp_immuno/final_results/pVACseq/mhc_i/10146-0054-TumorDNA.all_epitopes.tsv</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>/Volumes/gillandersw/Active/Project_0001_Clinical_Trials/CTEP/analysis/10146-CO070-0054/gcp_immuno/final_results/pVACseq/mhc_ii/10146-0054-TumorDNA.all_epitopes.aggregated.tsv</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>A Ward case was not included in the training set</t>
+        </is>
+      </c>
       <c r="I48" t="inlineStr">
         <is>
           <t>No</t>
@@ -3971,30 +3965,24 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K48" t="n">
-        <v>34</v>
-      </c>
-      <c r="L48" t="n">
-        <v>10</v>
-      </c>
-      <c r="M48" t="n">
-        <v>0</v>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr">
         <is>
-          <t>chr20-64105860-64105861-C-T</t>
+          <t>chr17-41505290-41505291-C-G</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>NPBWR2</t>
+          <t>KRT13</t>
         </is>
       </c>
       <c r="P48" t="n">
-        <v>0.482</v>
+        <v>0.498</v>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
@@ -4002,28 +3990,28 @@
         </is>
       </c>
       <c r="R48" t="n">
-        <v>0.964</v>
+        <v>0.996</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>04143-004</t>
+          <t>10146-0062</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SCLC</t>
+          <t>Metastatic TNBC</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Ward</t>
+          <t>CTEP</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>FAM135B,RB1,TP53</t>
+          <t>TP53,ACVR1B,ACVR2A,AKT2,APC,ATRX,BRAF,BRCA2,DAXX,ELF3,EP300,FAT1,FAT4,GNAS,HIF1A,KRAS,MAP2K4,MEN1,PREX2,RNF43,SMAD4,SND1,STK11</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
@@ -4031,7 +4019,7 @@
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
-          <t>A Ward case was not included in the training set</t>
+          <t xml:space="preserve"> Video analysis: after prediction revealed</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -4045,59 +4033,171 @@
         </is>
       </c>
       <c r="K49" t="n">
-        <v>158</v>
+        <v>58</v>
       </c>
       <c r="L49" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="M49" t="n">
         <v>0</v>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>chr17-41505290-41505291-C-G</t>
+          <t>chr17-7674946-7674947-A-G</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>KRT13</t>
+          <t>TP53</t>
         </is>
       </c>
       <c r="P49" t="n">
-        <v>0.498</v>
+        <v>0.485</v>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="R49" t="n">
-        <v>0.996</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr"/>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>TWJF-04143-005</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>SCLC</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Ward</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>FAM135B,RB1,TP53</t>
+        </is>
+      </c>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
-          <t> </t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr"/>
-      <c r="Q50" t="inlineStr"/>
-      <c r="R50" t="inlineStr"/>
+          <t>A Ward case was not included in the training set</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K50" t="n">
+        <v>157</v>
+      </c>
+      <c r="L50" t="n">
+        <v>18</v>
+      </c>
+      <c r="M50" t="n">
+        <v>0</v>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>chr21-32794112-32794113-C-G</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>C21orf62</t>
+        </is>
+      </c>
+      <c r="P50" t="n">
+        <v>0.498</v>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="R50" t="n">
+        <v>0.996</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>10146-0061</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Metastatic TNBC</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>CTEP</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>BARD1,BRCA2,RB1,TP53</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K51" t="n">
+        <v>221</v>
+      </c>
+      <c r="L51" t="n">
+        <v>50</v>
+      </c>
+      <c r="M51" t="n">
+        <v>0</v>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>chr17-7675075-7675076-T-C</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>TP53</t>
+        </is>
+      </c>
+      <c r="P51" t="n">
+        <v>0.484</v>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="R51" t="n">
+        <v>0.968</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>